<commit_message>
Added antenna cable to bill od materials
</commit_message>
<xml_diff>
--- a/JLCPCB Order/Bill of Materials.xlsx
+++ b/JLCPCB Order/Bill of Materials.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Client\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Client\Documents\GitHub\rfid-nfc-manager\JLCPCB Order\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{11182702-22C1-4817-8D7D-AB90B8DD381D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16BB713D-6689-4478-B8C2-7A038E6DEC2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="25800" windowHeight="15345" xr2:uid="{33F2DA52-EEA3-47B3-A567-6D5168423C5F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15480" xr2:uid="{33F2DA52-EEA3-47B3-A567-6D5168423C5F}"/>
   </bookViews>
   <sheets>
     <sheet name="RFID" sheetId="3" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="233">
   <si>
     <t>Reference</t>
   </si>
@@ -746,6 +746,12 @@
   </si>
   <si>
     <t>https://www.mouser.pl/en/ProductDetail/Texas-Instruments/BQ27441DRZT-G1A?qs=vvk%2Fphg2gmODra%2FNlpx9UQ%3D%3D</t>
+  </si>
+  <si>
+    <t>Anenna Connection Wires</t>
+  </si>
+  <si>
+    <t>https://www.mouser.pl/en/ProductDetail/Molex/15134-0301?qs=lQAVKuKFhkL4Aonld%2FWL2g%3D%3D</t>
   </si>
 </sst>
 </file>
@@ -754,7 +760,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;zł&quot;"/>
-    <numFmt numFmtId="170" formatCode="#,##0.000\ &quot;zł&quot;"/>
+    <numFmt numFmtId="165" formatCode="#,##0.000\ &quot;zł&quot;"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -800,22 +806,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -826,17 +828,17 @@
   <dxfs count="6">
     <dxf>
       <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;zł&quot;"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;zł&quot;"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="164" formatCode="#,##0.00\ &quot;zł&quot;"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -880,12 +882,12 @@
     <tableColumn id="1" xr3:uid="{F16D9625-9B1E-4AEB-9246-CDE52BA4BE12}" uniqueName="1" name="Reference" queryTableFieldId="1" dataDxfId="5"/>
     <tableColumn id="3" xr3:uid="{0CE96DDB-24C8-4DA3-BADA-AE7896D3402B}" uniqueName="3" name="Value" queryTableFieldId="3" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{913BA5DE-D16C-49E5-BCC5-928AE6C6536C}" uniqueName="2" name="Qty" queryTableFieldId="2"/>
-    <tableColumn id="6" xr3:uid="{5AA8CCA3-4938-44BC-86B7-1719F7D4981E}" uniqueName="6" name="Price" queryTableFieldId="6" dataDxfId="0"/>
-    <tableColumn id="7" xr3:uid="{009DB6CD-5A08-4ECD-8CC1-A6F04554B046}" uniqueName="7" name="Full Price" queryTableFieldId="7" dataDxfId="1">
+    <tableColumn id="6" xr3:uid="{5AA8CCA3-4938-44BC-86B7-1719F7D4981E}" uniqueName="6" name="Price" queryTableFieldId="6" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{009DB6CD-5A08-4ECD-8CC1-A6F04554B046}" uniqueName="7" name="Full Price" queryTableFieldId="7" dataDxfId="0">
       <calculatedColumnFormula>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{C5D5866C-93DB-43C2-906C-8763999F1784}" uniqueName="5" name="Name" queryTableFieldId="5" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{B3E4820C-7529-4EB8-8FDB-C30FFBA22F3F}" uniqueName="4" name="Site" queryTableFieldId="4" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{B3E4820C-7529-4EB8-8FDB-C30FFBA22F3F}" uniqueName="4" name="Site" queryTableFieldId="4" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1214,9 +1216,9 @@
     <col min="1" max="1" width="90.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="114.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.140625" style="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="26.85546875" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="150.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1230,13 +1232,13 @@
       <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="4" t="s">
         <v>184</v>
       </c>
       <c r="G1" t="s">
@@ -1244,1432 +1246,1438 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>4</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
-      <c r="D2" s="7">
+      <c r="D2" s="5">
         <v>10.039999999999999</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>10.039999999999999</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>7</v>
       </c>
       <c r="C3">
         <v>5</v>
       </c>
-      <c r="D3" s="8">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E3" s="4">
+      <c r="D3" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E3" s="3">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>1.8049999999999999</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>10</v>
       </c>
       <c r="C4">
         <v>4</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="6">
         <v>0.39900000000000002</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="3">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>1.5960000000000001</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>168</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>12</v>
       </c>
       <c r="C5">
         <v>21</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="6">
         <v>0.105</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="3">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>2.2050000000000001</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="G5" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>15</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="5">
         <v>1.41</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E6" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>1.41</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="G6" s="1" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>17</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="5">
         <v>1.08</v>
       </c>
-      <c r="E7" s="3">
+      <c r="E7" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>1.08</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G7" s="1" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="A8" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>20</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="5">
         <v>1.63</v>
       </c>
-      <c r="E8" s="3">
+      <c r="E8" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>1.63</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G8" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="A9" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>23</v>
       </c>
       <c r="C9">
         <v>2</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="6">
         <v>0.65100000000000002</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E9" s="3">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>1.302</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G9" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="A10" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>26</v>
       </c>
       <c r="C10">
         <v>1</v>
       </c>
-      <c r="D10" s="7">
+      <c r="D10" s="5">
         <v>0.5</v>
       </c>
-      <c r="E10" s="3">
+      <c r="E10" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>0.5</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="F10" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" s="1" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="A11" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>29</v>
       </c>
       <c r="C11">
         <v>2</v>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="6">
         <v>0.45400000000000001</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E11" s="3">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>0.90800000000000003</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="G11" s="1" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="A12" t="s">
         <v>169</v>
       </c>
-      <c r="B12" s="1"/>
       <c r="C12">
         <v>2</v>
       </c>
-      <c r="E12" s="3">
+      <c r="E12" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>0</v>
       </c>
-      <c r="F12" s="6"/>
-      <c r="G12" s="1" t="s">
+      <c r="G12" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="A13" t="s">
         <v>170</v>
       </c>
-      <c r="B13" s="1"/>
       <c r="C13">
         <v>2</v>
       </c>
-      <c r="E13" s="3">
+      <c r="E13" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>0</v>
       </c>
-      <c r="F13" s="6"/>
-      <c r="G13" s="1"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="A14" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>34</v>
       </c>
       <c r="C14">
         <v>2</v>
       </c>
-      <c r="D14" s="7">
+      <c r="D14" s="5">
         <v>1.08</v>
       </c>
-      <c r="E14" s="3">
+      <c r="E14" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>2.16</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="F14" s="4" t="s">
         <v>155</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="G14" s="1" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+      <c r="A15" t="s">
         <v>36</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" t="s">
         <v>37</v>
       </c>
       <c r="C15">
         <v>1</v>
       </c>
-      <c r="D15" s="8">
+      <c r="D15" s="6">
         <v>0.39900000000000002</v>
       </c>
-      <c r="E15" s="4">
+      <c r="E15" s="3">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>0.39900000000000002</v>
       </c>
-      <c r="F15" s="6" t="s">
+      <c r="F15" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="G15" s="1" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
+      <c r="A16" t="s">
         <v>39</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" t="s">
         <v>173</v>
       </c>
       <c r="C16">
         <v>1</v>
       </c>
-      <c r="D16" s="8">
+      <c r="D16" s="6">
         <v>0.83199999999999996</v>
       </c>
-      <c r="E16" s="4">
+      <c r="E16" s="3">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>0.83199999999999996</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="F16" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="G16" s="1" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+      <c r="A17" t="s">
         <v>40</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" t="s">
         <v>173</v>
       </c>
       <c r="C17">
         <v>3</v>
       </c>
-      <c r="D17" s="7">
+      <c r="D17" s="5">
         <v>2.39</v>
       </c>
-      <c r="E17" s="3">
+      <c r="E17" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>7.17</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="F17" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="G17" s="2" t="s">
+      <c r="G17" s="1" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
+      <c r="A18" t="s">
         <v>162</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" t="s">
         <v>173</v>
       </c>
       <c r="C18">
         <v>2</v>
       </c>
-      <c r="D18" s="7">
+      <c r="D18" s="5">
         <v>1.23</v>
       </c>
-      <c r="E18" s="3">
+      <c r="E18" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>2.46</v>
       </c>
-      <c r="F18" s="6">
+      <c r="F18" s="4">
         <v>824520600</v>
       </c>
-      <c r="G18" s="2" t="s">
+      <c r="G18" s="1" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+      <c r="A19" t="s">
         <v>43</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" t="s">
         <v>174</v>
       </c>
       <c r="C19">
         <v>1</v>
       </c>
-      <c r="D19" s="7">
+      <c r="D19" s="5">
         <v>1.1599999999999999</v>
       </c>
-      <c r="E19" s="3">
+      <c r="E19" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>1.1599999999999999</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="F19" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="G19" s="1" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+      <c r="A20" t="s">
         <v>45</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" t="s">
         <v>46</v>
       </c>
       <c r="C20">
         <v>1</v>
       </c>
-      <c r="D20" s="8">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E20" s="4">
-        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="F20" s="6" t="s">
+      <c r="D20" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E20" s="3">
+        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="F20" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="G20" s="2" t="s">
+      <c r="G20" s="1" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
+      <c r="A21" t="s">
         <v>163</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" t="s">
         <v>49</v>
       </c>
       <c r="C21">
         <v>2</v>
       </c>
-      <c r="D21" s="8">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E21" s="4">
+      <c r="D21" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E21" s="3">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>0.72199999999999998</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="F21" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="G21" s="2" t="s">
+      <c r="G21" s="1" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
+      <c r="A22" t="s">
         <v>50</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" t="s">
         <v>175</v>
       </c>
       <c r="C22">
         <v>5</v>
       </c>
-      <c r="D22" s="8">
+      <c r="D22" s="6">
         <v>1.5780000000000001</v>
       </c>
-      <c r="E22" s="3">
+      <c r="E22" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>7.8900000000000006</v>
       </c>
-      <c r="F22" s="6" t="s">
+      <c r="F22" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="G22" s="2" t="s">
+      <c r="G22" s="1" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
+      <c r="A23" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" t="s">
         <v>178</v>
       </c>
       <c r="C23">
         <v>5</v>
       </c>
-      <c r="D23" s="8">
+      <c r="D23" s="6">
         <v>6.5979999999999999</v>
       </c>
-      <c r="E23" s="3">
+      <c r="E23" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>32.99</v>
       </c>
-      <c r="F23" s="6" t="s">
+      <c r="F23" s="4" t="s">
         <v>177</v>
       </c>
-      <c r="G23" s="2" t="s">
+      <c r="G23" s="1" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
+      <c r="A24" t="s">
         <v>53</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" t="s">
         <v>180</v>
       </c>
       <c r="C24">
         <v>1</v>
       </c>
-      <c r="D24" s="7">
+      <c r="D24" s="5">
         <v>12.39</v>
       </c>
-      <c r="E24" s="3">
+      <c r="E24" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>12.39</v>
       </c>
-      <c r="F24" s="6" t="s">
+      <c r="F24" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="G24" s="2" t="s">
+      <c r="G24" s="1" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
+      <c r="A25" t="s">
         <v>54</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" t="s">
         <v>187</v>
       </c>
       <c r="C25">
         <v>1</v>
       </c>
-      <c r="D25" s="7">
+      <c r="D25" s="5">
         <v>4.45</v>
       </c>
-      <c r="E25" s="3">
+      <c r="E25" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>4.45</v>
       </c>
-      <c r="F25" s="6" t="s">
+      <c r="F25" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="G25" s="2" t="s">
+      <c r="G25" s="1" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
+      <c r="A26" t="s">
         <v>55</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" t="s">
         <v>190</v>
       </c>
       <c r="C26">
         <v>1</v>
       </c>
-      <c r="D26" s="7">
+      <c r="D26" s="5">
         <v>1.63</v>
       </c>
-      <c r="E26" s="3">
+      <c r="E26" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>1.63</v>
       </c>
-      <c r="F26" s="6" t="s">
+      <c r="F26" s="4" t="s">
         <v>189</v>
       </c>
-      <c r="G26" s="2" t="s">
+      <c r="G26" s="1" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
+      <c r="A27" t="s">
         <v>193</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" t="s">
         <v>194</v>
       </c>
       <c r="C27">
         <v>3</v>
       </c>
-      <c r="D27" s="7">
+      <c r="D27" s="5">
         <v>1.44</v>
       </c>
-      <c r="E27" s="3">
+      <c r="E27" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>4.32</v>
       </c>
-      <c r="F27" s="6" t="s">
+      <c r="F27" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="G27" s="2" t="s">
+      <c r="G27" s="1" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
+      <c r="A28" t="s">
         <v>56</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" t="s">
         <v>191</v>
       </c>
       <c r="C28">
         <v>1</v>
       </c>
-      <c r="D28" s="7">
+      <c r="D28" s="5">
         <v>1.7</v>
       </c>
-      <c r="E28" s="3">
+      <c r="E28" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>1.7</v>
       </c>
-      <c r="F28" s="6" t="s">
+      <c r="F28" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="G28" s="2" t="s">
+      <c r="G28" s="1" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
+      <c r="A29" t="s">
         <v>60</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B29" t="s">
         <v>7</v>
       </c>
       <c r="C29">
         <v>1</v>
       </c>
-      <c r="D29" s="8">
+      <c r="D29" s="6">
         <v>0.90300000000000002</v>
       </c>
-      <c r="E29" s="4">
+      <c r="E29" s="3">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>0.90300000000000002</v>
       </c>
-      <c r="F29" s="6" t="s">
+      <c r="F29" s="4" t="s">
         <v>196</v>
       </c>
-      <c r="G29" s="2" t="s">
+      <c r="G29" s="1" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
+      <c r="A30" t="s">
         <v>61</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B30" t="s">
         <v>62</v>
       </c>
       <c r="C30">
         <v>2</v>
       </c>
-      <c r="D30" s="8">
+      <c r="D30" s="6">
         <v>0.72199999999999998</v>
       </c>
-      <c r="E30" s="4">
+      <c r="E30" s="3">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>1.444</v>
       </c>
-      <c r="F30" s="6" t="s">
+      <c r="F30" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="G30" s="2" t="s">
+      <c r="G30" s="1" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
+      <c r="A31" t="s">
         <v>65</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B31" t="s">
         <v>66</v>
       </c>
       <c r="C31">
         <v>1</v>
       </c>
-      <c r="D31" s="7">
+      <c r="D31" s="5">
         <v>1.44</v>
       </c>
-      <c r="E31" s="3">
+      <c r="E31" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>1.44</v>
       </c>
-      <c r="F31" s="6" t="s">
+      <c r="F31" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="G31" s="2" t="s">
+      <c r="G31" s="1" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
+      <c r="A32" t="s">
         <v>67</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" t="s">
         <v>210</v>
       </c>
       <c r="C32">
         <v>1</v>
       </c>
-      <c r="D32" s="8">
+      <c r="D32" s="6">
         <v>0.72199999999999998</v>
       </c>
-      <c r="E32" s="4">
+      <c r="E32" s="3">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>0.72199999999999998</v>
       </c>
-      <c r="F32" s="6" t="s">
+      <c r="F32" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="G32" s="2" t="s">
+      <c r="G32" s="1" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
+      <c r="A33" t="s">
         <v>70</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" t="s">
         <v>211</v>
       </c>
       <c r="C33">
         <v>1</v>
       </c>
-      <c r="D33" s="8">
+      <c r="D33" s="6">
         <v>0.504</v>
       </c>
-      <c r="E33" s="4">
+      <c r="E33" s="3">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>0.504</v>
       </c>
-      <c r="F33" s="6" t="s">
+      <c r="F33" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="G33" s="2" t="s">
+      <c r="G33" s="1" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="1" t="s">
+      <c r="A34" t="s">
         <v>73</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" t="s">
         <v>212</v>
       </c>
       <c r="C34">
         <v>1</v>
       </c>
-      <c r="D34" s="8">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E34" s="4">
-        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="F34" s="6" t="s">
+      <c r="D34" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E34" s="3">
+        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="F34" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="G34" s="2" t="s">
+      <c r="G34" s="1" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="s">
+      <c r="A35" t="s">
         <v>74</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B35" t="s">
         <v>75</v>
       </c>
       <c r="C35">
         <v>1</v>
       </c>
-      <c r="D35" s="8">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E35" s="4">
-        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="F35" s="6" t="s">
+      <c r="D35" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E35" s="3">
+        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="F35" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="G35" s="2" t="s">
+      <c r="G35" s="1" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="1" t="s">
+      <c r="A36" t="s">
         <v>78</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" t="s">
         <v>79</v>
       </c>
       <c r="C36">
         <v>1</v>
       </c>
-      <c r="D36" s="8">
+      <c r="D36" s="6">
         <v>0.45400000000000001</v>
       </c>
-      <c r="E36" s="4">
+      <c r="E36" s="3">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>0.45400000000000001</v>
       </c>
-      <c r="F36" s="6" t="s">
+      <c r="F36" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="G36" s="2" t="s">
+      <c r="G36" s="1" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="1" t="s">
+      <c r="A37" t="s">
         <v>81</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="B37" t="s">
         <v>82</v>
       </c>
       <c r="C37">
         <v>1</v>
       </c>
-      <c r="D37" s="8">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E37" s="4">
-        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="F37" s="6" t="s">
+      <c r="D37" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E37" s="3">
+        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="F37" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="G37" s="2" t="s">
+      <c r="G37" s="1" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="1" t="s">
+      <c r="A38" t="s">
         <v>84</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B38" t="s">
         <v>85</v>
       </c>
       <c r="C38">
         <v>1</v>
       </c>
-      <c r="D38" s="8">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E38" s="4">
-        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="F38" s="6" t="s">
+      <c r="D38" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E38" s="3">
+        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="F38" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="G38" s="2" t="s">
+      <c r="G38" s="1" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" s="1" t="s">
+      <c r="A39" t="s">
         <v>88</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B39" t="s">
         <v>89</v>
       </c>
       <c r="C39">
         <v>1</v>
       </c>
-      <c r="D39" s="8">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E39" s="4">
-        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="F39" s="6" t="s">
+      <c r="D39" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E39" s="3">
+        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="F39" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="G39" s="2" t="s">
+      <c r="G39" s="1" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" s="1" t="s">
+      <c r="A40" t="s">
         <v>92</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="B40" t="s">
         <v>93</v>
       </c>
       <c r="C40">
         <v>2</v>
       </c>
-      <c r="D40" s="8">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E40" s="4">
+      <c r="D40" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E40" s="3">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>0.72199999999999998</v>
       </c>
-      <c r="F40" s="6" t="s">
+      <c r="F40" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="G40" s="2" t="s">
+      <c r="G40" s="1" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="1" t="s">
+      <c r="A41" t="s">
         <v>95</v>
       </c>
-      <c r="B41" s="1" t="s">
+      <c r="B41" t="s">
         <v>96</v>
       </c>
       <c r="C41">
         <v>2</v>
       </c>
-      <c r="D41" s="8">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E41" s="4">
+      <c r="D41" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E41" s="3">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>0.72199999999999998</v>
       </c>
-      <c r="F41" s="6" t="s">
+      <c r="F41" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="G41" s="2" t="s">
+      <c r="G41" s="1" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" s="1" t="s">
+      <c r="A42" t="s">
         <v>98</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="B42" t="s">
         <v>99</v>
       </c>
       <c r="C42">
         <v>5</v>
       </c>
-      <c r="D42" s="8">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E42" s="4">
+      <c r="D42" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E42" s="3">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>1.8049999999999999</v>
       </c>
-      <c r="F42" s="6" t="s">
+      <c r="F42" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="G42" s="2" t="s">
+      <c r="G42" s="1" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" s="1" t="s">
+      <c r="A43" t="s">
         <v>101</v>
       </c>
-      <c r="B43" s="1" t="s">
+      <c r="B43" t="s">
         <v>82</v>
       </c>
       <c r="C43">
         <v>1</v>
       </c>
-      <c r="D43" s="8">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E43" s="4">
-        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="F43" s="6" t="s">
+      <c r="D43" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E43" s="3">
+        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="F43" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="G43" s="2" t="s">
+      <c r="G43" s="1" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="1" t="s">
+      <c r="A44" t="s">
         <v>103</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="B44" t="s">
         <v>104</v>
       </c>
       <c r="C44">
         <v>1</v>
       </c>
-      <c r="D44" s="8">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E44" s="4">
-        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="F44" s="6" t="s">
+      <c r="D44" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E44" s="3">
+        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="F44" s="4" t="s">
         <v>202</v>
       </c>
-      <c r="G44" s="2" t="s">
+      <c r="G44" s="1" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A45" s="1" t="s">
+      <c r="A45" t="s">
         <v>106</v>
       </c>
-      <c r="B45" s="1" t="s">
+      <c r="B45" t="s">
         <v>107</v>
       </c>
       <c r="C45">
         <v>1</v>
       </c>
-      <c r="D45" s="8">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E45" s="4">
-        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="F45" s="6" t="s">
+      <c r="D45" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E45" s="3">
+        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="F45" s="4" t="s">
         <v>203</v>
       </c>
-      <c r="G45" s="2" t="s">
+      <c r="G45" s="1" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" s="1" t="s">
+      <c r="A46" t="s">
         <v>108</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="B46" t="s">
         <v>109</v>
       </c>
       <c r="C46">
         <v>1</v>
       </c>
-      <c r="D46" s="8">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E46" s="4">
-        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="F46" s="6" t="s">
+      <c r="D46" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E46" s="3">
+        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="F46" s="4" t="s">
         <v>204</v>
       </c>
-      <c r="G46" s="2" t="s">
+      <c r="G46" s="1" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="1" t="s">
+      <c r="A47" t="s">
         <v>119</v>
       </c>
-      <c r="B47" s="1"/>
       <c r="C47">
         <v>2</v>
       </c>
-      <c r="D47" s="8"/>
-      <c r="E47" s="3">
+      <c r="D47" s="6"/>
+      <c r="E47" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>0</v>
       </c>
-      <c r="F47" s="6"/>
-      <c r="G47" s="2"/>
+      <c r="G47" s="1"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="1" t="s">
+      <c r="A48" t="s">
         <v>111</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="B48" t="s">
         <v>112</v>
       </c>
       <c r="C48">
         <v>2</v>
       </c>
-      <c r="D48" s="8">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E48" s="4">
+      <c r="D48" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E48" s="3">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>0.72199999999999998</v>
       </c>
-      <c r="F48" s="6" t="s">
+      <c r="F48" s="4" t="s">
         <v>205</v>
       </c>
-      <c r="G48" s="2" t="s">
+      <c r="G48" s="1" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" s="1" t="s">
+      <c r="A49" t="s">
         <v>114</v>
       </c>
-      <c r="B49" s="1" t="s">
+      <c r="B49" t="s">
         <v>96</v>
       </c>
       <c r="C49">
         <v>1</v>
       </c>
-      <c r="D49" s="8">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E49" s="4">
-        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="F49" s="6" t="s">
+      <c r="D49" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E49" s="3">
+        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="F49" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="G49" s="2" t="s">
+      <c r="G49" s="1" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="1" t="s">
+      <c r="A50" t="s">
         <v>116</v>
       </c>
-      <c r="B50" s="1" t="s">
+      <c r="B50" t="s">
         <v>117</v>
       </c>
       <c r="C50">
         <v>1</v>
       </c>
-      <c r="D50" s="8">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E50" s="4">
-        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="F50" s="6" t="s">
+      <c r="D50" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E50" s="3">
+        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="F50" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="G50" s="2" t="s">
+      <c r="G50" s="1" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" s="1" t="s">
+      <c r="A51" t="s">
         <v>120</v>
       </c>
-      <c r="B51" s="1" t="s">
+      <c r="B51" t="s">
         <v>46</v>
       </c>
       <c r="C51">
         <v>4</v>
       </c>
-      <c r="D51" s="8">
-        <v>0.36099999999999999</v>
-      </c>
-      <c r="E51" s="4">
+      <c r="D51" s="6">
+        <v>0.36099999999999999</v>
+      </c>
+      <c r="E51" s="3">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>1.444</v>
       </c>
-      <c r="F51" s="6" t="s">
+      <c r="F51" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="G51" s="2" t="s">
+      <c r="G51" s="1" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" s="1" t="s">
+      <c r="A52" t="s">
         <v>122</v>
       </c>
-      <c r="B52" s="1" t="s">
+      <c r="B52" t="s">
         <v>123</v>
       </c>
       <c r="C52">
         <v>1</v>
       </c>
-      <c r="D52" s="8">
+      <c r="D52" s="6">
         <v>0.45400000000000001</v>
       </c>
-      <c r="E52" s="4">
+      <c r="E52" s="3">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>0.45400000000000001</v>
       </c>
-      <c r="F52" s="6" t="s">
+      <c r="F52" s="4" t="s">
         <v>222</v>
       </c>
-      <c r="G52" s="2" t="s">
+      <c r="G52" s="1" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" s="1" t="s">
+      <c r="A53" t="s">
         <v>125</v>
       </c>
-      <c r="B53" s="1" t="s">
+      <c r="B53" t="s">
         <v>126</v>
       </c>
       <c r="C53">
         <v>1</v>
       </c>
-      <c r="D53" s="7">
+      <c r="D53" s="5">
         <v>3.68</v>
       </c>
-      <c r="E53" s="3">
+      <c r="E53" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>3.68</v>
       </c>
-      <c r="F53" s="6" t="s">
+      <c r="F53" s="4" t="s">
         <v>218</v>
       </c>
-      <c r="G53" s="2" t="s">
+      <c r="G53" s="1" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A54" s="1" t="s">
+      <c r="A54" t="s">
         <v>128</v>
       </c>
-      <c r="B54" s="1" t="s">
+      <c r="B54" t="s">
         <v>223</v>
       </c>
       <c r="C54">
         <v>1</v>
       </c>
-      <c r="D54" s="7">
+      <c r="D54" s="5">
         <v>1.73</v>
       </c>
-      <c r="E54" s="3">
+      <c r="E54" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>1.73</v>
       </c>
-      <c r="F54" s="6" t="s">
+      <c r="F54" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="G54" s="2" t="s">
+      <c r="G54" s="1" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" s="1" t="s">
+      <c r="A55" t="s">
         <v>164</v>
       </c>
-      <c r="B55" s="1" t="s">
+      <c r="B55" t="s">
         <v>165</v>
       </c>
       <c r="C55">
         <v>2</v>
       </c>
-      <c r="D55" s="8">
+      <c r="D55" s="6">
         <v>0.54200000000000004</v>
       </c>
-      <c r="E55" s="4">
+      <c r="E55" s="3">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>1.0840000000000001</v>
       </c>
-      <c r="F55" s="6" t="s">
+      <c r="F55" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="G55" s="2" t="s">
+      <c r="G55" s="1" t="s">
         <v>224</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" s="1" t="s">
+      <c r="A56" t="s">
         <v>166</v>
       </c>
-      <c r="B56" s="1" t="s">
+      <c r="B56" t="s">
         <v>167</v>
       </c>
       <c r="C56">
         <v>2</v>
       </c>
-      <c r="D56" s="8">
+      <c r="D56" s="6">
         <v>0.504</v>
       </c>
-      <c r="E56" s="4">
+      <c r="E56" s="3">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>1.008</v>
       </c>
-      <c r="F56" s="6" t="s">
+      <c r="F56" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="G56" s="2" t="s">
+      <c r="G56" s="1" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="1" t="s">
+      <c r="A57" t="s">
         <v>134</v>
       </c>
-      <c r="B57" s="1" t="s">
+      <c r="B57" t="s">
         <v>99</v>
       </c>
       <c r="C57">
         <v>1</v>
       </c>
-      <c r="D57" s="7">
+      <c r="D57" s="5">
         <v>1.19</v>
       </c>
-      <c r="E57" s="3">
+      <c r="E57" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>1.19</v>
       </c>
-      <c r="F57" s="6" t="s">
+      <c r="F57" s="4" t="s">
         <v>219</v>
       </c>
-      <c r="G57" s="2" t="s">
+      <c r="G57" s="1" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" s="1" t="s">
+      <c r="A58" t="s">
         <v>136</v>
       </c>
-      <c r="B58" s="1" t="s">
+      <c r="B58" t="s">
         <v>228</v>
       </c>
       <c r="C58">
         <v>1</v>
       </c>
-      <c r="D58" s="7">
+      <c r="D58" s="5">
         <v>2.56</v>
       </c>
-      <c r="E58" s="3">
+      <c r="E58" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>2.56</v>
       </c>
-      <c r="F58" s="6" t="s">
+      <c r="F58" s="4" t="s">
         <v>226</v>
       </c>
-      <c r="G58" s="2" t="s">
+      <c r="G58" s="1" t="s">
         <v>225</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A59" s="1" t="s">
+      <c r="A59" t="s">
         <v>137</v>
       </c>
-      <c r="B59" s="1" t="s">
+      <c r="B59" t="s">
         <v>229</v>
       </c>
       <c r="C59">
         <v>1</v>
       </c>
-      <c r="D59" s="7">
+      <c r="D59" s="5">
         <v>12.64</v>
       </c>
-      <c r="E59" s="3">
+      <c r="E59" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>12.64</v>
       </c>
-      <c r="F59" s="6" t="s">
+      <c r="F59" s="4" t="s">
         <v>227</v>
       </c>
-      <c r="G59" s="2" t="s">
+      <c r="G59" s="1" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" s="1" t="s">
+      <c r="A60" t="s">
         <v>138</v>
       </c>
-      <c r="B60" s="1" t="s">
+      <c r="B60" t="s">
         <v>139</v>
       </c>
       <c r="C60">
         <v>1</v>
       </c>
-      <c r="D60" s="7">
+      <c r="D60" s="5">
         <v>4.01</v>
       </c>
-      <c r="E60" s="3">
+      <c r="E60" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>4.01</v>
       </c>
-      <c r="F60" s="6" t="s">
+      <c r="F60" s="4" t="s">
         <v>220</v>
       </c>
-      <c r="G60" s="2" t="s">
+      <c r="G60" s="1" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A61" s="1" t="s">
+      <c r="A61" t="s">
         <v>141</v>
       </c>
-      <c r="B61" s="1" t="s">
+      <c r="B61" t="s">
         <v>142</v>
       </c>
       <c r="C61">
         <v>1</v>
       </c>
-      <c r="D61" s="7">
+      <c r="D61" s="5">
         <v>2.13</v>
       </c>
-      <c r="E61" s="3">
+      <c r="E61" s="2">
         <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
         <v>2.13</v>
       </c>
-      <c r="F61" s="6" t="s">
+      <c r="F61" s="4" t="s">
         <v>221</v>
       </c>
-      <c r="G61" s="2" t="s">
+      <c r="G61" s="1" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A62" s="1"/>
-      <c r="B62" s="1"/>
-      <c r="F62" s="6"/>
-      <c r="G62" s="1"/>
+      <c r="A62" t="s">
+        <v>231</v>
+      </c>
+      <c r="C62">
+        <v>1</v>
+      </c>
+      <c r="D62" s="5">
+        <v>11.8</v>
+      </c>
+      <c r="E62" s="2">
+        <f>RFID__2[[#This Row],[Qty]]*RFID__2[[#This Row],[Price]]</f>
+        <v>11.8</v>
+      </c>
+      <c r="G62" t="s">
+        <v>232</v>
+      </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A63" s="1"/>
-      <c r="B63" s="1"/>
-      <c r="F63" s="6"/>
-      <c r="G63" s="2"/>
+      <c r="E63" s="2">
+        <f>SUM(E2:E62)</f>
+        <v>160.24900000000002</v>
+      </c>
+      <c r="G63" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>